<commit_message>
mage general install, myrm repal, ch 5d map, ch 5d dev
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -5799,10 +5799,820 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>UnitID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Lv</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Str</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mag</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Skl</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Spd</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Def</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Res</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Luck</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Con</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Hit</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Crit</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>AS</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dragon_Veteran</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>72</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="n">
+        <v>11</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>32</v>
+      </c>
+      <c r="N2" t="n">
+        <v>137</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dragon_Veteran</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" t="n">
+        <v>72</v>
+      </c>
+      <c r="D3" t="n">
+        <v>24</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G3" t="n">
+        <v>17</v>
+      </c>
+      <c r="H3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>37</v>
+      </c>
+      <c r="N3" t="n">
+        <v>132</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ch5Eagle_MageGeneral</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>34</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J4" t="n">
+        <v>14</v>
+      </c>
+      <c r="K4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>AblatioPhoton</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>31</v>
+      </c>
+      <c r="N4" t="n">
+        <v>172</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ch5Eagle_MageGeneral</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>34</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>19</v>
+      </c>
+      <c r="G5" t="n">
+        <v>20</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="n">
+        <v>17</v>
+      </c>
+      <c r="J5" t="n">
+        <v>14</v>
+      </c>
+      <c r="K5" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Elfire</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" t="n">
+        <v>147</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Storm_Myrmidon</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>34</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>14</v>
+      </c>
+      <c r="G6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SteelSword</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" t="n">
+        <v>111</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>UnitID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Lv</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Str</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mag</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Skl</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Spd</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Def</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Res</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Luck</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Con</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Hit</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Crit</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>AS</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dragon_Veteran</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>72</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="n">
+        <v>11</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>32</v>
+      </c>
+      <c r="N2" t="n">
+        <v>137</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dragon_Veteran</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" t="n">
+        <v>72</v>
+      </c>
+      <c r="D3" t="n">
+        <v>24</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G3" t="n">
+        <v>17</v>
+      </c>
+      <c r="H3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>37</v>
+      </c>
+      <c r="N3" t="n">
+        <v>132</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ch5Eagle_MageGeneral</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>34</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J4" t="n">
+        <v>14</v>
+      </c>
+      <c r="K4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>AblatioPhoton</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>31</v>
+      </c>
+      <c r="N4" t="n">
+        <v>172</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ch5Eagle_MageGeneral</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>34</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>19</v>
+      </c>
+      <c r="G5" t="n">
+        <v>20</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="n">
+        <v>17</v>
+      </c>
+      <c r="J5" t="n">
+        <v>14</v>
+      </c>
+      <c r="K5" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Elfire</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" t="n">
+        <v>147</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Storm_Myrmidon</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>34</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>14</v>
+      </c>
+      <c r="G6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SteelSword</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" t="n">
+        <v>111</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="4" customWidth="1" min="2" max="2"/>
     <col width="4" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
@@ -5814,10 +6624,10 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="5" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
-    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
     <col width="6" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
     <col width="7" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
@@ -6022,21 +6832,95 @@
         <v>39</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>JabberwockBoss_Jabberwock</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" t="n">
+        <v>57</v>
+      </c>
+      <c r="D4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Beast_Revenant</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="n">
+        <v>53</v>
+      </c>
+      <c r="D5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="4" customWidth="1" min="2" max="2"/>
     <col width="4" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
@@ -6048,10 +6932,10 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="5" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
-    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
     <col width="6" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
     <col width="7" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
@@ -6256,472 +7140,78 @@
         <v>39</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
-    <col width="5" customWidth="1" min="14" max="14"/>
-    <col width="6" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>UnitID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Lv</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>HP</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Str</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Mag</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Skl</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Spd</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Def</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Res</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Luck</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Con</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Weapon</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Atk</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Hit</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Crit</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>AS</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Dragon_Veteran</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" t="n">
-        <v>72</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24</v>
-      </c>
-      <c r="E2" t="n">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>JabberwockBoss_Jabberwock</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" t="n">
+        <v>57</v>
+      </c>
+      <c r="D4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Beast_Revenant</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="n">
+        <v>53</v>
+      </c>
+      <c r="D5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
         <v>3</v>
       </c>
-      <c r="F2" t="n">
-        <v>21</v>
-      </c>
-      <c r="G2" t="n">
-        <v>17</v>
-      </c>
-      <c r="H2" t="n">
-        <v>15</v>
-      </c>
-      <c r="I2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K2" t="n">
-        <v>11</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>IronLance</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>32</v>
-      </c>
-      <c r="N2" t="n">
-        <v>137</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Dragon_Veteran</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" t="n">
-        <v>72</v>
-      </c>
-      <c r="D3" t="n">
-        <v>24</v>
-      </c>
-      <c r="E3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F3" t="n">
-        <v>21</v>
-      </c>
-      <c r="G3" t="n">
-        <v>17</v>
-      </c>
-      <c r="H3" t="n">
-        <v>15</v>
-      </c>
-      <c r="I3" t="n">
-        <v>8</v>
-      </c>
-      <c r="J3" t="n">
-        <v>5</v>
-      </c>
-      <c r="K3" t="n">
-        <v>11</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>SteelBlade</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>37</v>
-      </c>
-      <c r="N3" t="n">
-        <v>132</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>39</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
-    <col width="5" customWidth="1" min="14" max="14"/>
-    <col width="6" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>UnitID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Lv</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>HP</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Str</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Mag</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Skl</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Spd</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Def</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Res</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Luck</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Con</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Weapon</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Atk</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Hit</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Crit</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>AS</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Dragon_Veteran</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" t="n">
-        <v>72</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24</v>
-      </c>
-      <c r="E2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F2" t="n">
-        <v>21</v>
-      </c>
-      <c r="G2" t="n">
-        <v>17</v>
-      </c>
-      <c r="H2" t="n">
-        <v>15</v>
-      </c>
-      <c r="I2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K2" t="n">
-        <v>11</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>IronLance</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>32</v>
-      </c>
-      <c r="N2" t="n">
-        <v>137</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Dragon_Veteran</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" t="n">
-        <v>72</v>
-      </c>
-      <c r="D3" t="n">
-        <v>24</v>
-      </c>
-      <c r="E3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F3" t="n">
-        <v>21</v>
-      </c>
-      <c r="G3" t="n">
-        <v>17</v>
-      </c>
-      <c r="H3" t="n">
-        <v>15</v>
-      </c>
-      <c r="I3" t="n">
-        <v>8</v>
-      </c>
-      <c r="J3" t="n">
-        <v>5</v>
-      </c>
-      <c r="K3" t="n">
-        <v>11</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>SteelBlade</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>37</v>
-      </c>
-      <c r="N3" t="n">
-        <v>132</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>39</v>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more ch 5 dev
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -1844,13 +1844,13 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="P18" s="2" t="n">
         <v>13</v>
@@ -7781,7 +7781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W57"/>
+  <dimension ref="A1:W59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11130,389 +11130,389 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Beast_Cyclops</t>
+          <t>Lowlander_Mercenary</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C49" s="4" t="n">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J49" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>SilverAxe</t>
+          <t>Lancereaver</t>
         </is>
       </c>
       <c r="M49" s="4" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O49" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P49" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q49" s="4" t="n">
         <v>31</v>
       </c>
       <c r="R49" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="S49" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="T49" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="U49" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="V49" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="S49" s="4" t="n">
-        <v>88</v>
-      </c>
-      <c r="T49" s="4" t="n">
-        <v>104</v>
-      </c>
-      <c r="U49" s="4" t="n">
-        <v>68</v>
-      </c>
-      <c r="V49" s="4" t="n">
-        <v>48</v>
-      </c>
       <c r="W49" s="4" t="n">
-        <v>64</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Beast_Jabberwock</t>
+          <t>Beast_Cyclops</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C50" s="4" t="n">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E50" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="H50" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J50" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I50" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J50" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K50" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>SilverAxe</t>
+        </is>
+      </c>
+      <c r="M50" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="N50" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="O50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L50" s="4" t="inlineStr">
-        <is>
-          <t>FetidClaw</t>
-        </is>
-      </c>
-      <c r="M50" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="N50" s="4" t="n">
-        <v>93</v>
-      </c>
-      <c r="O50" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P50" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="Q50" s="4" t="n">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="R50" s="4" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="S50" s="4" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="T50" s="4" t="n">
-        <v>58</v>
+        <v>104</v>
       </c>
       <c r="U50" s="4" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="V50" s="4" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="W50" s="4" t="n">
-        <v>29</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>0x87_MogallClass</t>
+          <t>Beast_Gargoyle</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C51" s="4" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G51" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="H51" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="H51" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="I51" s="4" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K51" s="4" t="n">
         <v>9</v>
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>EvilEye</t>
+          <t>SteelLance</t>
         </is>
       </c>
       <c r="M51" s="4" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="N51" s="4" t="n">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="O51" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P51" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q51" s="4" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R51" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S51" s="4" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="T51" s="4" t="n">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="U51" s="4" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="V51" s="4" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="W51" s="4" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>0x87_Bael</t>
+          <t>Beast_Jabberwock</t>
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E52" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J52" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" s="4" t="n">
         <v>15</v>
       </c>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>SharpClaw</t>
+          <t>FetidClaw</t>
         </is>
       </c>
       <c r="M52" s="4" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="N52" s="4" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="O52" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P52" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q52" s="4" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="R52" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="S52" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="T52" s="4" t="n">
         <v>58</v>
-      </c>
-      <c r="T52" s="4" t="n">
-        <v>65</v>
       </c>
       <c r="U52" s="4" t="n">
         <v>44</v>
       </c>
       <c r="V52" s="4" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="W52" s="4" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>0x87_Cyclops</t>
+          <t>0x87_MogallClass</t>
         </is>
       </c>
       <c r="B53" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C53" s="4" t="n">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="D53" s="4" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="G53" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I53" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="H53" s="4" t="n">
+      <c r="J53" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>EvilEye</t>
+        </is>
+      </c>
+      <c r="M53" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="I53" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="J53" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K53" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="L53" s="4" t="inlineStr">
-        <is>
-          <t>SharpClaw</t>
-        </is>
-      </c>
-      <c r="M53" s="4" t="n">
-        <v>38</v>
-      </c>
       <c r="N53" s="4" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="O53" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P53" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q53" s="4" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="R53" s="4" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="S53" s="4" t="n">
-        <v>95</v>
+        <v>54</v>
       </c>
       <c r="T53" s="4" t="n">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="U53" s="4" t="n">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="V53" s="4" t="n">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="W53" s="4" t="n">
-        <v>68</v>
+        <v>22</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>0x87_Revenant</t>
+          <t>0x87_Bael</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C54" s="4" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="D54" s="4" t="n">
         <v>17</v>
@@ -11521,22 +11521,22 @@
         <v>0</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H54" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J54" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I54" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J54" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K54" s="4" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
@@ -11547,218 +11547,218 @@
         <v>34</v>
       </c>
       <c r="N54" s="4" t="n">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="O54" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P54" s="4" t="n">
-        <v>-2</v>
+        <v>8</v>
       </c>
       <c r="Q54" s="4" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="R54" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="S54" s="4" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="T54" s="4" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="U54" s="4" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="V54" s="4" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="W54" s="4" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>0x87_Mercenary</t>
+          <t>0x87_Cyclops</t>
         </is>
       </c>
       <c r="B55" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C55" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>SharpClaw</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="N55" s="4" t="n">
+        <v>114</v>
+      </c>
+      <c r="O55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q55" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="D55" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E55" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="G55" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="H55" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I55" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J55" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K55" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="L55" s="4" t="inlineStr">
-        <is>
-          <t>SharpClaw</t>
-        </is>
-      </c>
-      <c r="M55" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="N55" s="4" t="n">
-        <v>106</v>
-      </c>
-      <c r="O55" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q55" s="4" t="n">
-        <v>29</v>
-      </c>
       <c r="R55" s="4" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="S55" s="4" t="n">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="T55" s="4" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="U55" s="4" t="n">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="V55" s="4" t="n">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="W55" s="4" t="n">
-        <v>22</v>
+        <v>68</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>0x87_LowMage</t>
+          <t>0x87_Revenant</t>
         </is>
       </c>
       <c r="B56" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C56" s="4" t="n">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="D56" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E56" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="F56" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="G56" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H56" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I56" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="J56" s="4" t="n">
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>SharpClaw</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="N56" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="O56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="4" t="n">
+        <v>-2</v>
+      </c>
+      <c r="Q56" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="R56" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K56" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>SharpClaw</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="N56" s="4" t="n">
-        <v>103</v>
-      </c>
-      <c r="O56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q56" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="R56" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="S56" s="4" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="T56" s="4" t="n">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="U56" s="4" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="V56" s="4" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="W56" s="4" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>0x87_Gargoyle</t>
+          <t>0x87_Mercenary</t>
         </is>
       </c>
       <c r="B57" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C57" s="4" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E57" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F57" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="G57" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="G57" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="H57" s="4" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I57" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J57" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K57" s="4" t="n">
         <v>9</v>
@@ -11769,36 +11769,186 @@
         </is>
       </c>
       <c r="M57" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="N57" s="4" t="n">
+        <v>106</v>
+      </c>
+      <c r="O57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q57" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="R57" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="S57" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="T57" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="U57" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="V57" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="W57" s="4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>0x87_LowMage</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C58" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="D58" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K58" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>SharpClaw</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="N58" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="O58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q58" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="R58" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S58" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="T58" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="U58" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="V58" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W58" s="4" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>0x87_Gargoyle</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="H59" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="I59" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>SharpClaw</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="N57" s="4" t="n">
+      <c r="N59" s="4" t="n">
         <v>101</v>
       </c>
-      <c r="O57" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P57" s="4" t="n">
+      <c r="O59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="Q57" s="4" t="n">
+      <c r="Q59" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="R57" s="4" t="n">
+      <c r="R59" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="S57" s="4" t="n">
+      <c r="S59" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="T57" s="4" t="n">
+      <c r="T59" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="U57" s="4" t="n">
+      <c r="U59" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="V57" s="4" t="n">
+      <c r="V59" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="W57" s="4" t="n">
+      <c r="W59" s="4" t="n">
         <v>35</v>
       </c>
     </row>
@@ -11813,7 +11963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W57"/>
+  <dimension ref="A1:W59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15162,46 +15312,46 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Beast_Cyclops</t>
+          <t>Lowlander_Mercenary</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I49" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C49" s="4" t="n">
-        <v>74</v>
-      </c>
-      <c r="D49" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="E49" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G49" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="H49" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="I49" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="J49" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>SilverAxe</t>
+          <t>Lancereaver</t>
         </is>
       </c>
       <c r="M49" s="4" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="N49" s="4" t="n">
         <v>110</v>
@@ -15210,209 +15360,209 @@
         <v>0</v>
       </c>
       <c r="P49" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Q49" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="R49" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S49" s="4" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="T49" s="4" t="n">
-        <v>96</v>
+        <v>35</v>
       </c>
       <c r="U49" s="4" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="V49" s="4" t="n">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="W49" s="4" t="n">
-        <v>59</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Beast_Jabberwock</t>
+          <t>Beast_Cyclops</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C50" s="4" t="n">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E50" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J50" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>FetidClaw</t>
+          <t>SilverAxe</t>
         </is>
       </c>
       <c r="M50" s="4" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="N50" s="4" t="n">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="O50" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P50" s="4" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="R50" s="4" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="S50" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="T50" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="U50" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="V50" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="W50" s="4" t="n">
         <v>59</v>
-      </c>
-      <c r="T50" s="4" t="n">
-        <v>58</v>
-      </c>
-      <c r="U50" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="V50" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="W50" s="4" t="n">
-        <v>29</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>0x87_MogallClass</t>
+          <t>Beast_Gargoyle</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C51" s="4" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H51" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K51" s="4" t="n">
         <v>9</v>
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>EvilEye</t>
+          <t>SteelLance</t>
         </is>
       </c>
       <c r="M51" s="4" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="N51" s="4" t="n">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="O51" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P51" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q51" s="4" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="R51" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="S51" s="4" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="T51" s="4" t="n">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="U51" s="4" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="V51" s="4" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="W51" s="4" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>0x87_Bael</t>
+          <t>Beast_Jabberwock</t>
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E52" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J52" s="4" t="n">
         <v>0</v>
@@ -15422,129 +15572,129 @@
       </c>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>SharpClaw</t>
+          <t>FetidClaw</t>
         </is>
       </c>
       <c r="M52" s="4" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="N52" s="4" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="O52" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P52" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q52" s="4" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="R52" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="S52" s="4" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="T52" s="4" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="U52" s="4" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="V52" s="4" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="W52" s="4" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>0x87_Cyclops</t>
+          <t>0x87_MogallClass</t>
         </is>
       </c>
       <c r="B53" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C53" s="4" t="n">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="D53" s="4" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="J53" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K53" s="4" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>SharpClaw</t>
+          <t>EvilEye</t>
         </is>
       </c>
       <c r="M53" s="4" t="n">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="N53" s="4" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="O53" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P53" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="Q53" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="R53" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S53" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="T53" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="U53" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="V53" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="R53" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="S53" s="4" t="n">
-        <v>88</v>
-      </c>
-      <c r="T53" s="4" t="n">
-        <v>104</v>
-      </c>
-      <c r="U53" s="4" t="n">
-        <v>68</v>
-      </c>
-      <c r="V53" s="4" t="n">
-        <v>48</v>
-      </c>
       <c r="W53" s="4" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>0x87_Revenant</t>
+          <t>0x87_Bael</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C54" s="4" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D54" s="4" t="n">
         <v>14</v>
@@ -15553,22 +15703,22 @@
         <v>0</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J54" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K54" s="4" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
@@ -15579,71 +15729,71 @@
         <v>31</v>
       </c>
       <c r="N54" s="4" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="O54" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P54" s="4" t="n">
-        <v>-3</v>
+        <v>7</v>
       </c>
       <c r="Q54" s="4" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="R54" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="S54" s="4" t="n">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="T54" s="4" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U54" s="4" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="V54" s="4" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="W54" s="4" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>0x87_Mercenary</t>
+          <t>0x87_Cyclops</t>
         </is>
       </c>
       <c r="B55" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C55" s="4" t="n">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="D55" s="4" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="E55" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J55" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
@@ -15651,146 +15801,146 @@
         </is>
       </c>
       <c r="M55" s="4" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="N55" s="4" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="O55" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P55" s="4" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="Q55" s="4" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="R55" s="4" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="S55" s="4" t="n">
-        <v>29</v>
+        <v>88</v>
       </c>
       <c r="T55" s="4" t="n">
-        <v>33</v>
+        <v>104</v>
       </c>
       <c r="U55" s="4" t="n">
-        <v>22</v>
+        <v>68</v>
       </c>
       <c r="V55" s="4" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="W55" s="4" t="n">
-        <v>19</v>
+        <v>64</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>0x87_LowMage</t>
+          <t>0x87_Revenant</t>
         </is>
       </c>
       <c r="B56" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C56" s="4" t="n">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="D56" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G56" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E56" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="F56" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G56" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="H56" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>SharpClaw</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="N56" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="O56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="4" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Q56" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R56" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K56" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>SharpClaw</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="N56" s="4" t="n">
-        <v>98</v>
-      </c>
-      <c r="O56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q56" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="R56" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="S56" s="4" t="n">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="T56" s="4" t="n">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="U56" s="4" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="V56" s="4" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="W56" s="4" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>0x87_Gargoyle</t>
+          <t>0x87_Mercenary</t>
         </is>
       </c>
       <c r="B57" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C57" s="4" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E57" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F57" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G57" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="G57" s="4" t="n">
-        <v>14</v>
-      </c>
       <c r="H57" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I57" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J57" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K57" s="4" t="n">
         <v>9</v>
@@ -15801,36 +15951,186 @@
         </is>
       </c>
       <c r="M57" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="N57" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q57" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="R57" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S57" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="T57" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="U57" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="V57" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="W57" s="4" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>0x87_LowMage</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C58" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="N57" s="4" t="n">
+      <c r="D58" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>SharpClaw</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="N58" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="O58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="R58" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S58" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="T58" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="U58" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="V58" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="W58" s="4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>0x87_Gargoyle</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H59" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="I59" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>SharpClaw</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="N59" s="4" t="n">
         <v>97</v>
       </c>
-      <c r="O57" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P57" s="4" t="n">
+      <c r="O59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="Q57" s="4" t="n">
+      <c r="Q59" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="R57" s="4" t="n">
+      <c r="R59" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="S57" s="4" t="n">
+      <c r="S59" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="T57" s="4" t="n">
+      <c r="T59" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="U57" s="4" t="n">
+      <c r="U59" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="V57" s="4" t="n">
+      <c r="V59" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="W57" s="4" t="n">
+      <c r="W59" s="4" t="n">
         <v>32</v>
       </c>
     </row>
@@ -18564,13 +18864,13 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="P18" s="2" t="n">
         <v>13</v>
@@ -31237,13 +31537,13 @@
         </is>
       </c>
       <c r="M26" s="3" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="P26" s="3" t="n">
         <v>13</v>
@@ -34299,13 +34599,13 @@
         </is>
       </c>
       <c r="M26" s="3" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="P26" s="3" t="n">
         <v>13</v>

</xml_diff>

<commit_message>
drop item issue fixed
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -5693,10 +5693,10 @@
         <v>12</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J50" s="4" t="n">
         <v>0</v>
@@ -5728,19 +5728,19 @@
         <v>12</v>
       </c>
       <c r="S50" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="T50" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="T50" s="4" t="n">
-        <v>55</v>
-      </c>
       <c r="U50" s="4" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="V50" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="W50" s="4" t="n">
         <v>25</v>
-      </c>
-      <c r="W50" s="4" t="n">
-        <v>33</v>
       </c>
     </row>
     <row r="51">
@@ -6306,26 +6306,26 @@
       </c>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>Armorslayer</t>
+          <t>SteelSword</t>
         </is>
       </c>
       <c r="M58" s="4" t="n">
         <v>24</v>
       </c>
       <c r="N58" s="4" t="n">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="O58" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P58" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q58" s="4" t="n">
         <v>22</v>
       </c>
       <c r="R58" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="S58" s="4" t="n">
         <v>42</v>
@@ -6456,26 +6456,26 @@
       </c>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>HeavySpear</t>
+          <t>SteelLance</t>
         </is>
       </c>
       <c r="M60" s="4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="N60" s="4" t="n">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="O60" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P60" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q60" s="4" t="n">
         <v>22</v>
       </c>
       <c r="R60" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S60" s="4" t="n">
         <v>42</v>
@@ -6521,7 +6521,7 @@
         <v>11</v>
       </c>
       <c r="I61" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J61" s="4" t="n">
         <v>1</v>
@@ -6553,16 +6553,16 @@
         <v>11</v>
       </c>
       <c r="S61" s="4" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="T61" s="4" t="n">
         <v>61</v>
       </c>
       <c r="U61" s="4" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="V61" s="4" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="W61" s="4" t="n">
         <v>36</v>
@@ -7121,7 +7121,7 @@
         <v>10</v>
       </c>
       <c r="I69" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J69" s="4" t="n">
         <v>0</v>
@@ -7153,16 +7153,16 @@
         <v>11</v>
       </c>
       <c r="S69" s="4" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="T69" s="4" t="n">
         <v>59</v>
       </c>
       <c r="U69" s="4" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="V69" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="W69" s="4" t="n">
         <v>34</v>
@@ -12916,10 +12916,10 @@
         <v>13</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J35" s="4" t="n">
         <v>0</v>
@@ -12951,19 +12951,19 @@
         <v>17</v>
       </c>
       <c r="S35" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="T35" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="T35" s="4" t="n">
-        <v>56</v>
-      </c>
       <c r="U35" s="4" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="V35" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="W35" s="4" t="n">
         <v>26</v>
-      </c>
-      <c r="W35" s="4" t="n">
-        <v>34</v>
       </c>
     </row>
     <row r="36">
@@ -15726,10 +15726,10 @@
         <v>11</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J35" s="4" t="n">
         <v>0</v>
@@ -15761,19 +15761,19 @@
         <v>15</v>
       </c>
       <c r="S35" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="T35" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="T35" s="4" t="n">
-        <v>51</v>
-      </c>
       <c r="U35" s="4" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="V35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="W35" s="4" t="n">
         <v>23</v>
-      </c>
-      <c r="W35" s="4" t="n">
-        <v>31</v>
       </c>
     </row>
     <row r="36">
@@ -27490,10 +27490,10 @@
         <v>14</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="J65" s="4" t="n">
         <v>0</v>
@@ -27525,19 +27525,19 @@
         <v>14</v>
       </c>
       <c r="S65" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="T65" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="T65" s="4" t="n">
-        <v>59</v>
-      </c>
       <c r="U65" s="4" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="V65" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="W65" s="4" t="n">
         <v>27</v>
-      </c>
-      <c r="W65" s="4" t="n">
-        <v>35</v>
       </c>
     </row>
     <row r="66">
@@ -27568,7 +27568,7 @@
         <v>11</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J66" s="4" t="n">
         <v>1</v>
@@ -27600,16 +27600,16 @@
         <v>12</v>
       </c>
       <c r="S66" s="4" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="T66" s="4" t="n">
         <v>65</v>
       </c>
       <c r="U66" s="4" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="V66" s="4" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="W66" s="4" t="n">
         <v>38</v>
@@ -32605,10 +32605,10 @@
         <v>12</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J65" s="4" t="n">
         <v>0</v>
@@ -32640,19 +32640,19 @@
         <v>12</v>
       </c>
       <c r="S65" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="T65" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="T65" s="4" t="n">
-        <v>53</v>
-      </c>
       <c r="U65" s="4" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="V65" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="W65" s="4" t="n">
         <v>24</v>
-      </c>
-      <c r="W65" s="4" t="n">
-        <v>32</v>
       </c>
     </row>
     <row r="66">
@@ -32683,7 +32683,7 @@
         <v>10</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J66" s="4" t="n">
         <v>0</v>
@@ -32715,16 +32715,16 @@
         <v>11</v>
       </c>
       <c r="S66" s="4" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="T66" s="4" t="n">
         <v>59</v>
       </c>
       <c r="U66" s="4" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="V66" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="W66" s="4" t="n">
         <v>34</v>
@@ -36771,10 +36771,10 @@
         <v>14</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="J50" s="4" t="n">
         <v>1</v>
@@ -36806,19 +36806,19 @@
         <v>14</v>
       </c>
       <c r="S50" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="T50" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="T50" s="4" t="n">
-        <v>61</v>
-      </c>
       <c r="U50" s="4" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="V50" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="W50" s="4" t="n">
         <v>29</v>
-      </c>
-      <c r="W50" s="4" t="n">
-        <v>37</v>
       </c>
     </row>
     <row r="51">
@@ -37384,26 +37384,26 @@
       </c>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>Armorslayer</t>
+          <t>SteelSword</t>
         </is>
       </c>
       <c r="M58" s="4" t="n">
         <v>27</v>
       </c>
       <c r="N58" s="4" t="n">
-        <v>124</v>
+        <v>104</v>
       </c>
       <c r="O58" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P58" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="Q58" s="4" t="n">
         <v>25</v>
       </c>
       <c r="R58" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S58" s="4" t="n">
         <v>48</v>
@@ -37534,26 +37534,26 @@
       </c>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>HeavySpear</t>
+          <t>SteelLance</t>
         </is>
       </c>
       <c r="M60" s="4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="N60" s="4" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="O60" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P60" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q60" s="4" t="n">
         <v>25</v>
       </c>
       <c r="R60" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S60" s="4" t="n">
         <v>48</v>
@@ -37599,7 +37599,7 @@
         <v>12</v>
       </c>
       <c r="I61" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J61" s="4" t="n">
         <v>2</v>
@@ -37631,16 +37631,16 @@
         <v>12</v>
       </c>
       <c r="S61" s="4" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="T61" s="4" t="n">
         <v>67</v>
       </c>
       <c r="U61" s="4" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="V61" s="4" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="W61" s="4" t="n">
         <v>39</v>
@@ -38199,7 +38199,7 @@
         <v>11</v>
       </c>
       <c r="I69" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J69" s="4" t="n">
         <v>1</v>
@@ -38231,16 +38231,16 @@
         <v>12</v>
       </c>
       <c r="S69" s="4" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="T69" s="4" t="n">
         <v>65</v>
       </c>
       <c r="U69" s="4" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="V69" s="4" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="W69" s="4" t="n">
         <v>38</v>

</xml_diff>

<commit_message>
baseconvos with old clib
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -1436,7 +1436,7 @@
         <v>10</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>11</v>
@@ -1451,7 +1451,7 @@
         <v>11</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>0</v>
@@ -1486,19 +1486,19 @@
         <v>15</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="W14" s="3" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15"/>
@@ -3243,7 +3243,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>12</v>
@@ -3258,7 +3258,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>1</v>
@@ -3293,19 +3293,19 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -3318,7 +3318,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>12</v>
@@ -3333,7 +3333,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>1</v>
@@ -3368,19 +3368,19 @@
         <v>8</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -9640,7 +9640,7 @@
         <v>10</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>11</v>
@@ -9655,7 +9655,7 @@
         <v>11</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>0</v>
@@ -9690,19 +9690,19 @@
         <v>15</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="W14" s="3" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15"/>
@@ -11447,7 +11447,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>12</v>
@@ -11462,7 +11462,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>1</v>
@@ -11497,19 +11497,19 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -11522,7 +11522,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>12</v>
@@ -11537,7 +11537,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>1</v>
@@ -11572,19 +11572,19 @@
         <v>8</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -14257,7 +14257,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>12</v>
@@ -14272,7 +14272,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>1</v>
@@ -14307,19 +14307,19 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -14332,7 +14332,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>12</v>
@@ -14347,7 +14347,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>1</v>
@@ -14382,19 +14382,19 @@
         <v>8</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -17067,7 +17067,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>12</v>
@@ -17082,7 +17082,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>1</v>
@@ -17117,19 +17117,19 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -17142,7 +17142,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>12</v>
@@ -17157,7 +17157,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>1</v>
@@ -17192,19 +17192,19 @@
         <v>8</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -20579,7 +20579,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>12</v>
@@ -20594,7 +20594,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>1</v>
@@ -20629,19 +20629,19 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -20654,7 +20654,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>12</v>
@@ -20669,7 +20669,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>1</v>
@@ -20704,19 +20704,19 @@
         <v>8</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -24091,7 +24091,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>12</v>
@@ -24106,7 +24106,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>1</v>
@@ -24141,19 +24141,19 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -24166,7 +24166,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>12</v>
@@ -24181,7 +24181,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>1</v>
@@ -24216,19 +24216,19 @@
         <v>8</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -29206,7 +29206,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>12</v>
@@ -29221,7 +29221,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>1</v>
@@ -29256,19 +29256,19 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -29281,7 +29281,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>12</v>
@@ -29296,7 +29296,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>1</v>
@@ -29331,19 +29331,19 @@
         <v>8</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -34321,7 +34321,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>12</v>
@@ -34336,7 +34336,7 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>1</v>
@@ -34371,19 +34371,19 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -34396,7 +34396,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>12</v>
@@ -34411,7 +34411,7 @@
         <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>1</v>
@@ -34446,19 +34446,19 @@
         <v>8</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
ch 5d dev, shikari fix, fields anim fix
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -7949,10 +7949,10 @@
         <v>9</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="J2" s="4" t="n">
         <v>0</v>
@@ -7968,19 +7968,19 @@
       <c r="Q2" s="4" t="n"/>
       <c r="R2" s="4" t="n"/>
       <c r="S2" s="4" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="T2" s="4" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="W2" s="4" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -8464,10 +8464,10 @@
         <v>9</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="J2" s="4" t="n">
         <v>0</v>
@@ -8483,19 +8483,19 @@
       <c r="Q2" s="4" t="n"/>
       <c r="R2" s="4" t="n"/>
       <c r="S2" s="4" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="T2" s="4" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="W2" s="4" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
ch 5d end event
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -7779,20 +7779,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="6" customWidth="1" min="13" max="13"/>
     <col width="6" customWidth="1" min="14" max="14"/>
@@ -7925,361 +7925,716 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>0x80_CivMan</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3" t="n"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3" t="n"/>
+      <c r="R2" s="3" t="n"/>
+      <c r="S2" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>0x80_CivWoman</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
+      <c r="N3" s="3" t="n"/>
+      <c r="O3" s="3" t="n"/>
+      <c r="P3" s="3" t="n"/>
+      <c r="Q3" s="3" t="n"/>
+      <c r="R3" s="3" t="n"/>
+      <c r="S3" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="U3" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>0x80_CivGirl</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="U4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>0x80_CivBoy</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
+      <c r="N5" s="3" t="n"/>
+      <c r="O5" s="3" t="n"/>
+      <c r="P5" s="3" t="n"/>
+      <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="3" t="n"/>
+      <c r="S5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Veteran</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3" t="n"/>
+      <c r="P6" s="3" t="n"/>
+      <c r="Q6" s="3" t="n"/>
+      <c r="R6" s="3" t="n"/>
+      <c r="S6" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="T6" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="U6" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>0x82_Bard</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="n"/>
+      <c r="O7" s="3" t="n"/>
+      <c r="P7" s="3" t="n"/>
+      <c r="Q7" s="3" t="n"/>
+      <c r="R7" s="3" t="n"/>
+      <c r="S7" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="T7" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="U7" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>JabberwockBoss_Jabberwock</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" s="4" t="n">
+      <c r="B9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="4" t="n">
+      <c r="D9" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H2" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I2" s="4" t="n">
+      <c r="H9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I9" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="4" t="n">
+      <c r="J9" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="K9" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n">
+      <c r="L9" s="4" t="n"/>
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="n"/>
+      <c r="R9" s="4" t="n"/>
+      <c r="S9" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="T9" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="U2" s="4" t="n">
+      <c r="U9" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="V2" s="4" t="n">
+      <c r="V9" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="W9" s="4" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>JabberwockBlocker_Revenant</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="n">
+      <c r="B10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G3" s="4" t="n">
+      <c r="D10" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="K10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>RottenClaw</t>
         </is>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="N10" s="4" t="n">
         <v>107</v>
       </c>
-      <c r="O3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="4" t="n">
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="Q3" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="R3" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="S3" s="4" t="n">
+      <c r="Q10" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="T10" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="U10" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="V3" s="4" t="n">
+      <c r="V10" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="W3" s="4" t="n">
+      <c r="W10" s="4" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>JabberwockBlocker_BowBone</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C4" s="4" t="n">
+      <c r="B11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4" t="n">
+      <c r="D11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="H4" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="I4" s="4" t="n">
+      <c r="H11" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="I11" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="K11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Longbow</t>
         </is>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N11" s="4" t="n">
         <v>108</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q4" s="4" t="n">
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q11" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="R11" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S11" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="T11" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="U11" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="V4" s="4" t="n">
+      <c r="V11" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="W4" s="4" t="n">
+      <c r="W11" s="4" t="n">
         <v>23</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>JabberwockSiege_MogallClass</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C5" s="4" t="n">
+      <c r="B12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D12" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H5" s="4" t="n">
+      <c r="F12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Shadowshot</t>
         </is>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="M12" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="N12" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="O12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="P5" s="4" t="n">
+      <c r="P12" s="4" t="n">
         <v>-3</v>
       </c>
-      <c r="Q5" s="4" t="n">
+      <c r="Q12" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="R5" s="4" t="n">
+      <c r="R12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S5" s="4" t="n">
+      <c r="S12" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="T5" s="4" t="n">
+      <c r="T12" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="U5" s="4" t="n">
+      <c r="U12" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="V5" s="4" t="n">
+      <c r="V12" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="W5" s="4" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="W12" s="4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>JabberwockAttacker_Mauthedoog</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C6" s="4" t="n">
+      <c r="B13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D13" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="E6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="n">
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G13" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="H6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I6" s="4" t="n">
+      <c r="H13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J13" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="K13" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>FireFang</t>
         </is>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="M13" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N13" s="4" t="n">
         <v>159</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="4" t="n">
+      <c r="O13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="Q13" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="R13" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="S13" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="T13" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="U6" s="4" t="n">
+      <c r="U13" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="V6" s="4" t="n">
+      <c r="V13" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="W6" s="4" t="n">
+      <c r="W13" s="4" t="n">
         <v>22</v>
       </c>
     </row>
@@ -8294,20 +8649,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="6" customWidth="1" min="13" max="13"/>
     <col width="6" customWidth="1" min="14" max="14"/>
@@ -8440,361 +8795,716 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>0x80_CivMan</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3" t="n"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3" t="n"/>
+      <c r="R2" s="3" t="n"/>
+      <c r="S2" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>0x80_CivWoman</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
+      <c r="N3" s="3" t="n"/>
+      <c r="O3" s="3" t="n"/>
+      <c r="P3" s="3" t="n"/>
+      <c r="Q3" s="3" t="n"/>
+      <c r="R3" s="3" t="n"/>
+      <c r="S3" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="U3" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>0x80_CivGirl</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="U4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>0x80_CivBoy</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
+      <c r="N5" s="3" t="n"/>
+      <c r="O5" s="3" t="n"/>
+      <c r="P5" s="3" t="n"/>
+      <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="3" t="n"/>
+      <c r="S5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Veteran</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3" t="n"/>
+      <c r="P6" s="3" t="n"/>
+      <c r="Q6" s="3" t="n"/>
+      <c r="R6" s="3" t="n"/>
+      <c r="S6" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="T6" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="U6" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>0x82_Bard</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="n"/>
+      <c r="O7" s="3" t="n"/>
+      <c r="P7" s="3" t="n"/>
+      <c r="Q7" s="3" t="n"/>
+      <c r="R7" s="3" t="n"/>
+      <c r="S7" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="T7" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="U7" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>JabberwockBoss_Jabberwock</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" s="4" t="n">
+      <c r="B9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="4" t="n">
+      <c r="D9" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H2" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I2" s="4" t="n">
+      <c r="H9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I9" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="4" t="n">
+      <c r="J9" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="K9" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n">
+      <c r="L9" s="4" t="n"/>
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="n"/>
+      <c r="R9" s="4" t="n"/>
+      <c r="S9" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="T9" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="U2" s="4" t="n">
+      <c r="U9" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="V2" s="4" t="n">
+      <c r="V9" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="W9" s="4" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>JabberwockBlocker_Revenant</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="n">
+      <c r="B10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="4" t="n">
+      <c r="D10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="4" t="n">
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>RottenClaw</t>
         </is>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="N10" s="4" t="n">
         <v>104</v>
       </c>
-      <c r="O3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="4" t="n">
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="Q3" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="R3" s="4" t="n">
+      <c r="Q10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="S10" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="T10" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="U10" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="V3" s="4" t="n">
+      <c r="V10" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="W3" s="4" t="n">
+      <c r="W10" s="4" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>JabberwockBlocker_BowBone</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C4" s="4" t="n">
+      <c r="B11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4" t="n">
+      <c r="D11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="G4" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="I4" s="4" t="n">
+      <c r="G11" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I11" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Longbow</t>
         </is>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N11" s="4" t="n">
         <v>103</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q4" s="4" t="n">
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="R11" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S11" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="T11" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="U11" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="V4" s="4" t="n">
+      <c r="V11" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="W4" s="4" t="n">
+      <c r="W11" s="4" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>JabberwockSiege_MogallClass</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E5" s="4" t="n">
+      <c r="B12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Shadowshot</t>
         </is>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="M12" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="N12" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="O12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="P5" s="4" t="n">
+      <c r="P12" s="4" t="n">
         <v>-4</v>
       </c>
-      <c r="Q5" s="4" t="n">
+      <c r="Q12" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="R5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="4" t="n">
+      <c r="R12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="T5" s="4" t="n">
+      <c r="T12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="U5" s="4" t="n">
+      <c r="U12" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="V5" s="4" t="n">
+      <c r="V12" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="W5" s="4" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="W12" s="4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>JabberwockAttacker_Mauthedoog</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C6" s="4" t="n">
+      <c r="B13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D13" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="E6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="n">
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G13" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="K13" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>FireFang</t>
         </is>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="M13" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N13" s="4" t="n">
         <v>152</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="4" t="n">
+      <c r="O13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="Q13" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="R13" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="S13" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="T13" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="U6" s="4" t="n">
+      <c r="U13" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="V6" s="4" t="n">
+      <c r="V13" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="W6" s="4" t="n">
+      <c r="W13" s="4" t="n">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ch 6 start event
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -10611,26 +10611,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:Y25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="5" customWidth="1" min="14" max="14"/>
-    <col width="5" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
     <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
     <col width="7" customWidth="1" min="18" max="18"/>
     <col width="6" customWidth="1" min="19" max="19"/>
     <col width="6" customWidth="1" min="20" max="20"/>
@@ -10769,82 +10769,1821 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Soldier</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="R2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="T2" s="3" t="n"/>
+      <c r="U2" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Soldier</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q3" s="3" t="n">
+        <v>-4</v>
+      </c>
+      <c r="R3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="S3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="3" t="n"/>
+      <c r="U3" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Fighter</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Fighter</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="T5" s="3" t="n"/>
+      <c r="U5" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>0x82_LanceCav</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="T6" s="3" t="n"/>
+      <c r="U6" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y6" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>0x82_LanceCav</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="S7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" s="3" t="n"/>
+      <c r="U7" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y7" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>0x81_AxeCav</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="S8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="T8" s="3" t="n"/>
+      <c r="U8" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="V8" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="W8" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="X8" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y8" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>0x81_AxeCav</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="S9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="T9" s="3" t="n"/>
+      <c r="U9" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="W9" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y9" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Lion_Mage</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="T10" s="3" t="n"/>
+      <c r="U10" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="V10" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="W10" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y10" s="3" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Lion_Mage</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="S11" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="T11" s="3" t="n"/>
+      <c r="U11" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="W11" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y11" s="3" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>0x81_Mercenary</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C13" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D13" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="4" t="n">
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="G2" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="H2" s="4" t="n">
+      <c r="G13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J13" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K2" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="K13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>IronSword</t>
         </is>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="N13" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="O13" s="4" t="n">
         <v>136</v>
       </c>
-      <c r="P2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="R2" s="4" t="n">
+      <c r="P13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R13" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="S13" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n">
+      <c r="T13" s="4" t="n"/>
+      <c r="U13" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="V2" s="4" t="n">
+      <c r="V13" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="W13" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="X2" s="4" t="n">
+      <c r="X13" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="Y2" s="4" t="n">
+      <c r="Y13" s="4" t="n">
         <v>25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Skull_Fighter</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="T14" s="4" t="n"/>
+      <c r="U14" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="V14" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="W14" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="X14" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y14" s="4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Skull_Fighter</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T15" s="4" t="n"/>
+      <c r="U15" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="V15" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="W15" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="X15" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y15" s="4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>0x82_Brigand</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>94</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R16" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="S16" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="T16" s="4" t="n"/>
+      <c r="U16" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="V16" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="W16" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="X16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y16" s="4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>0x82_Brigand</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="O17" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="P17" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="S17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T17" s="4" t="n"/>
+      <c r="U17" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="V17" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="W17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="X17" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y17" s="4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>0x83_Mercenary</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R18" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S18" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="T18" s="4" t="n"/>
+      <c r="U18" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V18" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W18" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="X18" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y18" s="4" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>0x83_Mercenary</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="O19" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="P19" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R19" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S19" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T19" s="4" t="n"/>
+      <c r="U19" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V19" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W19" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="X19" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y19" s="4" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>0x84_Fighter</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T20" s="4" t="n"/>
+      <c r="U20" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="V20" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="W20" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="X20" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y20" s="4" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>0x84_Fighter</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="O21" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="P21" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S21" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T21" s="4" t="n"/>
+      <c r="U21" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="V21" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="W21" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="X21" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y21" s="4" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>0x84_CivMan</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>-2</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T22" s="4" t="n"/>
+      <c r="U22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="V22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="W22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="X22" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y22" s="4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>0x84_CivMan</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="P23" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q23" s="4" t="n">
+        <v>-10</v>
+      </c>
+      <c r="R23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="4" t="n">
+        <v>-6</v>
+      </c>
+      <c r="T23" s="4" t="n"/>
+      <c r="U23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="V23" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="W23" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="X23" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y23" s="4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>0x84_Mercenary</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="P24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R24" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S24" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="T24" s="4" t="n"/>
+      <c r="U24" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V24" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W24" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="X24" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y24" s="4" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>0x84_Mercenary</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="O25" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="P25" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q25" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R25" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S25" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T25" s="4" t="n"/>
+      <c r="U25" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V25" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W25" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="X25" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y25" s="4" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -10858,26 +12597,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:Y25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="5" customWidth="1" min="14" max="14"/>
-    <col width="5" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
     <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
     <col width="7" customWidth="1" min="18" max="18"/>
     <col width="6" customWidth="1" min="19" max="19"/>
     <col width="6" customWidth="1" min="20" max="20"/>
@@ -11016,82 +12755,1821 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Soldier</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="R2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="T2" s="3" t="n"/>
+      <c r="U2" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Soldier</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q3" s="3" t="n">
+        <v>-4</v>
+      </c>
+      <c r="R3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="S3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="3" t="n"/>
+      <c r="U3" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Fighter</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>0x81_Fighter</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="T5" s="3" t="n"/>
+      <c r="U5" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>0x82_LanceCav</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="T6" s="3" t="n"/>
+      <c r="U6" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y6" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>0x82_LanceCav</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="S7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" s="3" t="n"/>
+      <c r="U7" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y7" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>0x81_AxeCav</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="S8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="T8" s="3" t="n"/>
+      <c r="U8" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="V8" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="W8" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="X8" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y8" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>0x81_AxeCav</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="S9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="T9" s="3" t="n"/>
+      <c r="U9" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="W9" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y9" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Lion_Mage</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="T10" s="3" t="n"/>
+      <c r="U10" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="V10" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="W10" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y10" s="3" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Lion_Mage</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="S11" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="T11" s="3" t="n"/>
+      <c r="U11" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="W11" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y11" s="3" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>0x81_Mercenary</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C13" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="4" t="n">
+      <c r="D13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="G2" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" s="4" t="n">
+      <c r="G13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K2" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="K13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>IronSword</t>
         </is>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="N13" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="O13" s="4" t="n">
         <v>128</v>
       </c>
-      <c r="P2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="R2" s="4" t="n">
+      <c r="P13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="R13" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="S13" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n">
+      <c r="T13" s="4" t="n"/>
+      <c r="U13" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="V2" s="4" t="n">
+      <c r="V13" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="W13" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="X2" s="4" t="n">
+      <c r="X13" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="Y2" s="4" t="n">
+      <c r="Y13" s="4" t="n">
         <v>21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Skull_Fighter</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="T14" s="4" t="n"/>
+      <c r="U14" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="V14" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="W14" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="X14" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y14" s="4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Skull_Fighter</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T15" s="4" t="n"/>
+      <c r="U15" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="V15" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="W15" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="X15" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y15" s="4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>0x82_Brigand</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>94</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R16" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="S16" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="T16" s="4" t="n"/>
+      <c r="U16" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="V16" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="W16" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="X16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y16" s="4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>0x82_Brigand</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="O17" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="P17" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="S17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T17" s="4" t="n"/>
+      <c r="U17" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="V17" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="W17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="X17" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y17" s="4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>0x83_Mercenary</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R18" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S18" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="T18" s="4" t="n"/>
+      <c r="U18" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V18" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W18" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="X18" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y18" s="4" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>0x83_Mercenary</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="O19" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="P19" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R19" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S19" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T19" s="4" t="n"/>
+      <c r="U19" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V19" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W19" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="X19" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y19" s="4" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>0x84_Fighter</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T20" s="4" t="n"/>
+      <c r="U20" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="V20" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="W20" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="X20" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y20" s="4" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>0x84_Fighter</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="O21" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="P21" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S21" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T21" s="4" t="n"/>
+      <c r="U21" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="V21" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="W21" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="X21" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y21" s="4" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>0x84_CivMan</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>-2</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T22" s="4" t="n"/>
+      <c r="U22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="V22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="W22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="X22" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y22" s="4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>0x84_CivMan</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="P23" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q23" s="4" t="n">
+        <v>-10</v>
+      </c>
+      <c r="R23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="4" t="n">
+        <v>-6</v>
+      </c>
+      <c r="T23" s="4" t="n"/>
+      <c r="U23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="V23" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="W23" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="X23" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y23" s="4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>0x84_Mercenary</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>IronLance</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="P24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R24" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S24" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="T24" s="4" t="n"/>
+      <c r="U24" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V24" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W24" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="X24" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y24" s="4" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>0x84_Mercenary</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>SteelBlade</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="O25" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="P25" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q25" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R25" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S25" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T25" s="4" t="n"/>
+      <c r="U25" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V25" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="W25" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="X25" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y25" s="4" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ch 6 main events done
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -12372,7 +12372,7 @@
         <v>10</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
@@ -15148,7 +15148,7 @@
         <v>10</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
installing baby anim (incomplete)
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -2796,7 +2796,7 @@
         <v>15</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>40</v>
@@ -2875,7 +2875,7 @@
         <v>9</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="U3" s="2" t="n">
         <v>40</v>
@@ -2954,7 +2954,7 @@
         <v>15</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="U4" s="2" t="n">
         <v>40</v>
@@ -3337,7 +3337,7 @@
         <v>8</v>
       </c>
       <c r="T9" s="2" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U9" s="2" t="n">
         <v>47</v>
@@ -3572,7 +3572,7 @@
         <v>12</v>
       </c>
       <c r="T12" s="2" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="U12" s="2" t="n">
         <v>36</v>
@@ -3730,7 +3730,7 @@
         <v>18</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="U14" s="2" t="n">
         <v>37</v>
@@ -4032,7 +4032,7 @@
         <v>9</v>
       </c>
       <c r="T18" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="U18" s="2" t="n">
         <v>36</v>
@@ -4111,7 +4111,7 @@
         <v>14</v>
       </c>
       <c r="T19" s="2" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="U19" s="2" t="n">
         <v>36</v>
@@ -4579,7 +4579,7 @@
         <v>16</v>
       </c>
       <c r="T25" s="2" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="U25" s="2" t="n">
         <v>47</v>
@@ -5234,7 +5234,7 @@
         <v>11</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H35" s="3" t="n">
         <v>8</v>
@@ -5253,26 +5253,26 @@
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>SteelAxe</t>
+          <t>IronAxe</t>
         </is>
       </c>
       <c r="N35" s="3" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="P35" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S35" s="3" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="T35" s="3" t="n"/>
       <c r="U35" s="3" t="n">
@@ -52863,7 +52863,7 @@
         <v>15</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>40</v>
@@ -52942,7 +52942,7 @@
         <v>9</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="U3" s="2" t="n">
         <v>40</v>
@@ -53098,7 +53098,7 @@
         <v>16</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="U5" s="2" t="n">
         <v>35</v>
@@ -53177,7 +53177,7 @@
         <v>16</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="U6" s="2" t="n">
         <v>35</v>
@@ -53256,7 +53256,7 @@
         <v>16</v>
       </c>
       <c r="T7" s="2" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="U7" s="2" t="n">
         <v>35</v>
@@ -53637,7 +53637,7 @@
         <v>12</v>
       </c>
       <c r="T12" s="2" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="U12" s="2" t="n">
         <v>36</v>
@@ -53716,7 +53716,7 @@
         <v>12</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="U13" s="2" t="n">
         <v>36</v>
@@ -53941,7 +53941,7 @@
         <v>8</v>
       </c>
       <c r="T16" s="2" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="U16" s="2" t="n">
         <v>42</v>
@@ -54411,7 +54411,7 @@
         <v>15</v>
       </c>
       <c r="T22" s="2" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="U22" s="2" t="n">
         <v>34</v>
@@ -54644,7 +54644,7 @@
         <v>16</v>
       </c>
       <c r="T25" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="U25" s="2" t="n">
         <v>47</v>
@@ -54800,7 +54800,7 @@
         <v>19</v>
       </c>
       <c r="T27" s="2" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="U27" s="2" t="n">
         <v>44</v>
@@ -55299,7 +55299,7 @@
         <v>13</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H35" s="3" t="n">
         <v>9</v>
@@ -55318,26 +55318,26 @@
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>SteelAxe</t>
+          <t>IronAxe</t>
         </is>
       </c>
       <c r="N35" s="3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="P35" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="S35" s="3" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="T35" s="3" t="n"/>
       <c r="U35" s="3" t="n">

</xml_diff>

<commit_message>
ch 7 ending editing
</commit_message>
<xml_diff>
--- a/unit_stats.xlsx
+++ b/unit_stats.xlsx
@@ -21640,7 +21640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y22"/>
+  <dimension ref="A1:Y23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21913,7 +21913,7 @@
         <v>9</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
@@ -23099,7 +23099,7 @@
         <v>8</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
@@ -23376,6 +23376,85 @@
       </c>
       <c r="Y22" s="4" t="n">
         <v>25</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>0x81_Druid</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="P23" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="R23" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="S23" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="T23" s="4" t="n"/>
+      <c r="U23" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="V23" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="W23" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="X23" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y23" s="4" t="n">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -23389,7 +23468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y22"/>
+  <dimension ref="A1:Y23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -23662,7 +23741,7 @@
         <v>9</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
@@ -24848,7 +24927,7 @@
         <v>8</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
@@ -25125,6 +25204,85 @@
       </c>
       <c r="Y22" s="4" t="n">
         <v>22</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>0x81_Druid</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>128</v>
+      </c>
+      <c r="P23" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q23" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="R23" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="S23" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="T23" s="4" t="n"/>
+      <c r="U23" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="V23" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="W23" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="X23" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="Y23" s="4" t="n">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>